<commit_message>
Update StickerBinStickersCosts.xlsx with new cost data and adjustments
</commit_message>
<xml_diff>
--- a/stikerts/StickerBinStickersCosts.xlsx
+++ b/stikerts/StickerBinStickersCosts.xlsx
@@ -1,20 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4af2e227e45ba049/Documents/stikerts/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\liron\Local Sites\ordermachine\app\public\wp-content\plugins\orderMachine\stikerts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="23" documentId="11_9A9F6AFFB1F4D40AB5AA634FA848C3F19135DDE4" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{83159E95-7E92-4265-BCF1-D447552E3946}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{215D1C48-1E8B-4FEA-B248-99990C701833}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tier 1 Equipment Costs" sheetId="1" r:id="rId1"/>
     <sheet name="Bin Stickers 100x150 4pk" sheetId="2" r:id="rId2"/>
+    <sheet name="Montly expense" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
@@ -34,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="113">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="120">
   <si>
     <t>Bin Stickers — 100×140mm, 4-Pack (1 A4 sheet) — Cost Breakdown</t>
   </si>
@@ -373,6 +374,27 @@
   </si>
   <si>
     <t>Total</t>
+  </si>
+  <si>
+    <t>name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cost </t>
+  </si>
+  <si>
+    <t>details</t>
+  </si>
+  <si>
+    <t>lovart</t>
+  </si>
+  <si>
+    <t>Midjerny</t>
+  </si>
+  <si>
+    <t>accounting</t>
+  </si>
+  <si>
+    <t>total</t>
   </si>
 </sst>
 </file>
@@ -677,10 +699,6 @@
 </styleSheet>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -1713,4 +1731,61 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{32C45B9E-4755-413B-B4E9-4EAF3F254B63}">
+  <dimension ref="A1:C14"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="9.88671875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>113</v>
+      </c>
+      <c r="B1" t="s">
+        <v>114</v>
+      </c>
+      <c r="C1" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>116</v>
+      </c>
+      <c r="B2">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>117</v>
+      </c>
+      <c r="B3">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>118</v>
+      </c>
+      <c r="B4">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>119</v>
+      </c>
+      <c r="B14">
+        <f>SUM(B2:B13)</f>
+        <v>60</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>